<commit_message>
Update reports 2026-10-27 10:06
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-10-27.xlsx
+++ b/gex_pivot_levels_2026-10-27.xlsx
@@ -15,12 +15,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Pivots" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NQ'!$A$1:$G$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RTY'!$A$1:$G$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NQ'!$A$1:$G$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RTY'!$A$1:$G$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CL'!$A$1:$G$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'GC'!$A$1:$G$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$53</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -532,228 +532,224 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>7601.43</v>
+        <v>7648.73</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>753</v>
+        <v>7600</v>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>-$8.01M</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>+$9.12M</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>7671.64</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>760</v>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>-$17.82M</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>+$17.98M</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>-$27.74M</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>+$35.33M</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="n">
-        <v>7648.73</v>
-      </c>
-      <c r="B3" s="5" t="n">
-        <v>7600</v>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>7688.73</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>7640</v>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>-$8.58M</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>+$9.77M</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>-$14.79M</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>+$17.88M</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>7653.73</v>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>7605</v>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>-$3.08M</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>+$3.99M</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>7688.73</v>
+        <v>7691.7</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>7640</v>
+        <v>762</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>-$74.43M</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>+$102.36M</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>7693.73</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>7645</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>-$14.79M</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>+$17.88M</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>-$8.33M</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>+$10.72M</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>7698.73</v>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>7650</v>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>-$21.99M</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>+$53.03M</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="n">
-        <v>7691.7</v>
-      </c>
-      <c r="B6" s="5" t="n">
-        <v>762</v>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7701.73</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>763</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>-$24.41M</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>+$38.61M</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>7693.73</v>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>7645</v>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>-$8.33M</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>+$10.72M</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>-$9.07M</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>+$37.12M</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="n">
-        <v>7698.73</v>
-      </c>
-      <c r="B8" s="5" t="n">
-        <v>7650</v>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>-$21.99M</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>+$53.03M</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
@@ -771,12 +767,12 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>-$6.98M</t>
+          <t>-$7.06M</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>+$12.41M</t>
+          <t>+$12.55M</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -804,12 +800,12 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>-$14.36M</t>
+          <t>-$14.68M</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>+$20.78M</t>
+          <t>+$21.24M</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -824,35 +820,35 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="5" t="n">
         <v>7721.79</v>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" s="5" t="n">
         <v>765</v>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>+$9.42M</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>+$22.60M</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>-$41.31M</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>+$116.17M</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -870,12 +866,12 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>-$3.07M</t>
+          <t>-$3.13M</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>+$36.85M</t>
+          <t>+$37.63M</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -886,73 +882,77 @@
       <c r="G12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="n">
+      <c r="A13" s="2" t="n">
+        <v>7731.82</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>766</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>+$6.15M</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>+$58.24M</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
         <v>7741.85</v>
       </c>
-      <c r="B13" s="5" t="n">
+      <c r="B14" s="5" t="n">
         <v>767</v>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>-$127.05M</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>+$147.43M</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>-$82.68M</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>+$173.13M</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>7748.73</v>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>7700</v>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>+$213.03K</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>+$25.73M</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>7768.73</v>
+        <v>7748.73</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>7720</v>
+        <v>7700</v>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
@@ -961,56 +961,147 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>+$12.13M</t>
+          <t>+$391.67K</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>+$14.30M</t>
+          <t>+$26.59M</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
+        <v>7751.88</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>768</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>+$32.73M</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>+$53.34M</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>7768.73</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>7720</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>+$12.39M</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>+$14.60M</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>7771.94</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>770</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>+$28.81M</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>+$41.63M</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
         <v>7773.73</v>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B19" s="2" t="n">
         <v>7725</v>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>+$2.32M</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>+$16.82M</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr"/>
+      <c r="G19" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G16"/>
+  <autoFilter ref="A1:G19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1022,7 +1113,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1085,12 +1176,12 @@
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>-$2.95M</t>
+          <t>-$5.90M</t>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>+$3.40M</t>
+          <t>+$6.56M</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
@@ -1106,218 +1197,226 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
+        <v>28985.65</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>701</v>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>-$1.52M</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>+$1.93M</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
         <v>29150.06</v>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B4" s="5" t="n">
         <v>705</v>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>+$89.17K</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>+$4.65M</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>29232.27</v>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>707</v>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>+$425.53K</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>+$1.96M</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>-$5.50M</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>+$10.72M</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>29272.6</v>
+        <v>29191.16</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>29100</v>
+        <v>706</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>-$14.64K</t>
+          <t>-$1.83M</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>+$108.31K</t>
+          <t>+$5.28M</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>29314.47</v>
+        <v>29272.6</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>709</v>
+        <v>29100</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>-$14.64K</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>+$108.31K</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>29273.37</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>708</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>-$1.69M</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>+$4.90M</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>-$8.05M</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>+$16.24M</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="n">
-        <v>29355.57</v>
-      </c>
-      <c r="B7" s="5" t="n">
-        <v>710</v>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>+$10.82M</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>+$18.63M</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>29372.6</v>
+        <v>29314.47</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>29200</v>
+        <v>709</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>+$59.72K</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>-$3.31M</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>+$144.03K</t>
+          <t>+$15.70M</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>29432.6</v>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>29260</v>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>-$80.79K</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>+$87.82K</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="A9" s="5" t="n">
+        <v>29355.57</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>710</v>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>-$7.60M</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>+$32.31M</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -1325,130 +1424,138 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>29437.78</v>
+        <v>29372.6</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>712</v>
+        <v>29200</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>-$129.35K</t>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>+$59.72K</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>+$3.10M</t>
+          <t>+$144.03K</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>29442.6</v>
+        <v>29396.68</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>29270</v>
+        <v>711</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>+$7.03K</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>-$2.00M</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>+$112.41K</t>
+          <t>+$23.29M</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G11" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>29452.6</v>
+        <v>29432.6</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>29280</v>
+        <v>29260</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>+$3.51K</t>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>-$80.79K</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>+$207.26K</t>
+          <t>+$87.82K</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>29472.6</v>
+        <v>29437.78</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>29300</v>
+        <v>712</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>+$17.56K</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>-$11.30M</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>+$207.26K</t>
+          <t>+$21.42M</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>29522.6</v>
+        <v>29442.6</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>29350</v>
+        <v>29270</v>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
@@ -1457,12 +1564,12 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>+$80.79K</t>
+          <t>+$7.03K</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>+$137.00K</t>
+          <t>+$112.41K</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -1473,77 +1580,69 @@
       <c r="G14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="n">
-        <v>29561.09</v>
-      </c>
-      <c r="B15" s="5" t="n">
-        <v>715</v>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>+$4.91M</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>+$9.42M</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="A15" s="2" t="n">
+        <v>29452.6</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>29280</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>+$3.51K</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>+$207.26K</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="n">
-        <v>29572.6</v>
-      </c>
-      <c r="B16" s="5" t="n">
-        <v>29400</v>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="A16" s="2" t="n">
+        <v>29472.6</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>29300</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>+$727.15K</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>+$881.71K</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>+$17.56K</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>+$207.26K</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>29602.19</v>
+        <v>29519.98</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
@@ -1552,78 +1651,70 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>+$473.90K</t>
+          <t>+$5.18M</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>+$2.12M</t>
+          <t>+$27.36M</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="n">
-        <v>29725.5</v>
-      </c>
-      <c r="B18" s="5" t="n">
-        <v>719</v>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>+$9.86M</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>+$13.55M</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="A18" s="2" t="n">
+        <v>29522.6</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>29350</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>+$80.79K</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>+$137.00K</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
-        <v>29848.81</v>
+        <v>29572.6</v>
       </c>
       <c r="B19" s="5" t="n">
-        <v>722</v>
+        <v>29400</v>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>-$1.29M</t>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>+$727.15K</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>+$5.23M</t>
+          <t>+$881.71K</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -1633,16 +1724,16 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="n">
-        <v>29972.12</v>
+        <v>29766.6</v>
       </c>
       <c r="B20" s="5" t="n">
-        <v>725</v>
+        <v>720</v>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
@@ -1651,12 +1742,12 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>+$3.24M</t>
+          <t>+$11.19M</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>+$3.84M</t>
+          <t>+$16.42M</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -1670,70 +1761,8 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
-        <v>30136.53</v>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>729</v>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>-$232.18K</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>+$558.22K</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>30383.14</v>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>735</v>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>+$2.05M</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>+$2.10M</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G22"/>
+  <autoFilter ref="A1:G20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1745,7 +1774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1795,33 +1824,33 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="n">
-        <v>2766.5</v>
-      </c>
-      <c r="B2" s="5" t="n">
-        <v>275</v>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="A2" s="2" t="n">
+        <v>2776.56</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>276</v>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>-$5.80M</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>+$11.03M</t>
-        </is>
-      </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>-$8.56M</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>+$20.46M</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -1829,43 +1858,39 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>2806.74</v>
+        <v>2786.62</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>+$3.86M</t>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>-$4.20M</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>+$4.06M</t>
+          <t>+$27.78M</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>2826.86</v>
+        <v>2816.8</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -1874,12 +1899,12 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>+$726.59K</t>
+          <t>+$8.51M</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>+$766.98K</t>
+          <t>+$9.45M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -1889,45 +1914,78 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>2836.92</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>282</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>+$1.76M</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>+$1.78M</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="5" t="n">
+    <row r="6">
+      <c r="A6" s="5" t="n">
         <v>2846.98</v>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B6" s="5" t="n">
         <v>283</v>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>+$7.95M</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>+$7.96M</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>+$8.03M</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>+$8.04M</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G5"/>
+  <autoFilter ref="A1:G6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2381,7 +2439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2455,12 +2513,12 @@
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>-$127.05M</t>
+          <t>-$82.68M</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>+$147.43M</t>
+          <t>+$173.13M</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
@@ -2481,24 +2539,24 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>7698.73</v>
+        <v>7721.79</v>
       </c>
       <c r="C3" s="5" t="n">
-        <v>7650</v>
+        <v>765</v>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>-$21.99M</t>
+          <t>-$41.31M</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>+$53.03M</t>
+          <t>+$116.17M</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
@@ -2531,12 +2589,12 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>-$24.41M</t>
+          <t>-$74.43M</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>+$38.61M</t>
+          <t>+$102.36M</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -2557,32 +2615,36 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>7723.73</v>
+        <v>7731.82</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>7675</v>
+        <v>766</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>-$3.07M</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>+$6.15M</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>+$36.85M</t>
+          <t>+$58.24M</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -2591,146 +2653,142 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>7748.73</v>
+        <v>7751.88</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>7700</v>
+        <v>768</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>+$32.73M</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>+$53.34M</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>7698.73</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>7650</v>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>+$213.03K</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>+$25.73M</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>-$21.99M</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>+$53.03M</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>7771.94</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>770</v>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>+$28.81M</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>+$41.63M</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
-        <v>7721.79</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>765</v>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>+$9.42M</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>+$22.60M</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="n">
-        <v>7708.73</v>
-      </c>
-      <c r="C8" s="5" t="n">
-        <v>7660</v>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="B9" s="2" t="n">
+        <v>7723.73</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>7675</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>-$14.36M</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>+$20.78M</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n">
-        <v>29355.57</v>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>710</v>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>+$10.82M</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>+$18.63M</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>-$3.13M</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>+$37.63M</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -2739,10 +2797,10 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>7601.43</v>
+        <v>7701.73</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>753</v>
+        <v>763</v>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
@@ -2751,168 +2809,164 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>-$17.82M</t>
+          <t>-$9.07M</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>+$17.98M</t>
+          <t>+$37.12M</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>7671.64</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>760</v>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>-$27.74M</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>+$35.33M</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n">
-        <v>7688.73</v>
-      </c>
-      <c r="C11" s="5" t="n">
-        <v>7640</v>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>-$14.79M</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>+$17.88M</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>29355.57</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>710</v>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>-$7.60M</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>+$32.31M</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>7773.73</v>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>7725</v>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>+$2.32M</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>+$16.82M</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>7768.73</v>
+        <v>2786.62</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>7720</v>
+        <v>277</v>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>+$12.13M</t>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>-$4.20M</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>+$14.30M</t>
+          <t>+$27.78M</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B14" s="5" t="n">
-        <v>29725.5</v>
-      </c>
-      <c r="C14" s="5" t="n">
-        <v>719</v>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="B14" s="2" t="n">
+        <v>29519.98</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>714</v>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>+$9.86M</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>+$13.55M</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>+$5.18M</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>+$27.36M</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -2921,184 +2975,180 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>7703.73</v>
+        <v>7748.73</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>7655</v>
+        <v>7700</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>-$6.98M</t>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>+$391.67K</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>+$12.41M</t>
+          <t>+$26.59M</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>29396.68</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>711</v>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>-$2.00M</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>+$23.29M</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>29437.78</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>712</v>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>-$11.30M</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>+$21.42M</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>7708.73</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>7660</v>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>-$14.68M</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>+$21.24M</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>RTY</t>
         </is>
       </c>
-      <c r="B16" s="5" t="n">
-        <v>2766.5</v>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>275</v>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="B19" s="2" t="n">
+        <v>2776.56</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>276</v>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>-$5.80M</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>+$11.03M</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="n">
-        <v>4031.87</v>
-      </c>
-      <c r="C17" s="5" t="n">
-        <v>368</v>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>+$8.45M</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>+$10.91M</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>7693.73</v>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>7645</v>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>-$8.33M</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>+$10.72M</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>-$8.56M</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>+$20.46M</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="n">
-        <v>7648.73</v>
-      </c>
-      <c r="C19" s="5" t="n">
-        <v>7600</v>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>-$8.58M</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>+$9.77M</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -3107,28 +3157,28 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>29561.09</v>
+        <v>7688.73</v>
       </c>
       <c r="C20" s="5" t="n">
-        <v>715</v>
+        <v>7640</v>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>+$4.91M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>-$14.79M</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>+$9.42M</t>
+          <t>+$17.88M</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
@@ -3138,73 +3188,69 @@
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="n">
-        <v>2846.98</v>
-      </c>
-      <c r="C21" s="5" t="n">
-        <v>283</v>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E21" s="9" t="inlineStr">
-        <is>
-          <t>+$7.95M</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>+$7.96M</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>7773.73</v>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>7725</v>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>+$2.32M</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>+$16.82M</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>100.04</v>
+        <v>29766.6</v>
       </c>
       <c r="C22" s="5" t="n">
-        <v>165</v>
+        <v>720</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>USO</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>+$4.35M</t>
+          <t>+$11.19M</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>+$5.90M</t>
+          <t>+$16.42M</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -3219,38 +3265,38 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B23" s="5" t="n">
-        <v>29848.81</v>
-      </c>
-      <c r="C23" s="5" t="n">
-        <v>722</v>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="B23" s="2" t="n">
+        <v>29273.37</v>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>708</v>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>-$1.29M</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>+$5.23M</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>-$8.05M</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>+$16.24M</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -3275,12 +3321,12 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>-$1.69M</t>
+          <t>-$3.31M</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>+$4.90M</t>
+          <t>+$15.70M</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -3290,69 +3336,73 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>29150.06</v>
+        <v>7768.73</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>705</v>
+        <v>7720</v>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>+$89.17K</t>
+          <t>+$12.39M</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>+$4.65M</t>
+          <t>+$14.60M</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>2806.74</v>
+        <v>7703.73</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>279</v>
+        <v>7655</v>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>+$3.86M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>-$7.06M</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>+$4.06M</t>
+          <t>+$12.55M</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
@@ -3367,76 +3417,76 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>4031.87</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>368</v>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>+$8.45M</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>+$10.91M</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n">
-        <v>7653.73</v>
-      </c>
-      <c r="C27" s="2" t="n">
-        <v>7605</v>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="B28" s="2" t="n">
+        <v>7693.73</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>7645</v>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>-$3.08M</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>+$3.99M</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>-$8.33M</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>+$10.72M</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="n">
-        <v>29972.12</v>
-      </c>
-      <c r="C28" s="5" t="n">
-        <v>725</v>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E28" s="9" t="inlineStr">
-        <is>
-          <t>+$3.24M</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>+$3.84M</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -3449,10 +3499,10 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>28944.55</v>
+        <v>29150.06</v>
       </c>
       <c r="C29" s="5" t="n">
-        <v>700</v>
+        <v>705</v>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
@@ -3461,12 +3511,12 @@
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>-$2.95M</t>
+          <t>-$5.50M</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>+$3.40M</t>
+          <t>+$10.72M</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
@@ -3483,28 +3533,28 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>29437.78</v>
+        <v>2816.8</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>712</v>
+        <v>280</v>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>-$129.35K</t>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr">
+        <is>
+          <t>+$8.51M</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>+$3.10M</t>
+          <t>+$9.45M</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -3514,107 +3564,107 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>29602.19</v>
+        <v>7648.73</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>716</v>
+        <v>7600</v>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>+$473.90K</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>-$8.01M</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>+$2.12M</t>
+          <t>+$9.12M</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="n">
-        <v>30383.14</v>
-      </c>
-      <c r="C32" s="2" t="n">
-        <v>735</v>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E32" s="8" t="inlineStr">
-        <is>
-          <t>+$2.05M</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>+$2.10M</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr"/>
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>2846.98</v>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>283</v>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>+$8.03M</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>+$8.04M</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>3999</v>
+        <v>28944.55</v>
       </c>
       <c r="C33" s="5" t="n">
-        <v>365</v>
+        <v>700</v>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>-$1.85M</t>
+          <t>-$5.90M</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>+$2.06M</t>
+          <t>+$6.56M</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
@@ -3629,106 +3679,106 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>100.04</v>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>165</v>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>+$4.35M</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>+$5.90M</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n">
-        <v>29232.27</v>
-      </c>
-      <c r="C34" s="2" t="n">
-        <v>707</v>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="B35" s="2" t="n">
+        <v>29191.16</v>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>706</v>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>+$425.53K</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>+$1.96M</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>-$1.83M</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>+$5.28M</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H34" s="3" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr">
         <is>
           <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="n">
-        <v>4178.12</v>
-      </c>
-      <c r="C35" s="5" t="n">
-        <v>84</v>
-      </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="inlineStr">
-        <is>
-          <t>-$1.41M</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="inlineStr">
-        <is>
-          <t>+$1.47M</t>
-        </is>
-      </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H35" s="6" t="inlineStr">
-        <is>
-          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>93.98</v>
+        <v>3999</v>
       </c>
       <c r="C36" s="5" t="n">
-        <v>155</v>
+        <v>365</v>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>USO</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>-$1.32M</t>
+          <t>-$1.85M</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>+$1.37M</t>
+          <t>+$2.06M</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
@@ -3745,96 +3795,104 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>97.01000000000001</v>
+        <v>28985.65</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>160</v>
+        <v>701</v>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>-$709.84K</t>
+          <t>-$1.52M</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>+$1.27M</t>
+          <t>+$1.93M</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>103.08</v>
+        <v>2836.92</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>170</v>
+        <v>282</v>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t>+$809.97K</t>
+          <t>+$1.76M</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>+$974.83K</t>
+          <t>+$1.78M</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>29572.6</v>
+        <v>4178.12</v>
       </c>
       <c r="C39" s="5" t="n">
-        <v>29400</v>
+        <v>84</v>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E39" s="9" t="inlineStr">
-        <is>
-          <t>+$727.15K</t>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>-$1.41M</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>+$881.71K</t>
+          <t>+$1.47M</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
@@ -3844,43 +3902,43 @@
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="n">
-        <v>2826.86</v>
-      </c>
-      <c r="C40" s="2" t="n">
-        <v>281</v>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>+$726.59K</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>+$766.98K</t>
-        </is>
-      </c>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="inlineStr">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>93.98</v>
+      </c>
+      <c r="C40" s="5" t="n">
+        <v>155</v>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>-$1.32M</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>+$1.37M</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -3889,66 +3947,62 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>30136.53</v>
+        <v>97.01000000000001</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>729</v>
+        <v>160</v>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>USO</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>-$232.18K</t>
+          <t>-$709.84K</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>+$558.22K</t>
+          <t>+$1.27M</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H41" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>4078.64</v>
+        <v>103.08</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>82</v>
+        <v>170</v>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>-$202.18K</t>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>+$809.97K</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>+$352.22K</t>
+          <t>+$974.83K</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
@@ -3961,28 +4015,28 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>3730.47</v>
+        <v>29572.6</v>
       </c>
       <c r="C43" s="5" t="n">
-        <v>75</v>
+        <v>29400</v>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E43" s="7" t="inlineStr">
-        <is>
-          <t>-$252.09K</t>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>+$727.15K</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>+$252.09K</t>
+          <t>+$881.71K</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
@@ -3992,35 +4046,35 @@
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>29452.6</v>
+        <v>4078.64</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>29280</v>
+        <v>82</v>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>+$3.51K</t>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>-$202.18K</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>+$207.26K</t>
+          <t>+$352.22K</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
@@ -4031,38 +4085,42 @@
       <c r="H44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="n">
-        <v>29472.6</v>
-      </c>
-      <c r="C45" s="2" t="n">
-        <v>29300</v>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>+$17.56K</t>
-        </is>
-      </c>
-      <c r="F45" s="3" t="inlineStr">
-        <is>
-          <t>+$207.26K</t>
-        </is>
-      </c>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H45" s="3" t="inlineStr"/>
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>3730.47</v>
+      </c>
+      <c r="C45" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>-$252.09K</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>+$252.09K</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -4071,10 +4129,10 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>29372.6</v>
+        <v>29452.6</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>29200</v>
+        <v>29280</v>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
@@ -4083,12 +4141,12 @@
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t>+$59.72K</t>
+          <t>+$3.51K</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>+$144.03K</t>
+          <t>+$207.26K</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
@@ -4105,10 +4163,10 @@
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>29522.6</v>
+        <v>29472.6</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>29350</v>
+        <v>29300</v>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
@@ -4117,12 +4175,12 @@
       </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
-          <t>+$80.79K</t>
+          <t>+$17.56K</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>+$137.00K</t>
+          <t>+$207.26K</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
@@ -4139,10 +4197,10 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>29442.6</v>
+        <v>29372.6</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>29270</v>
+        <v>29200</v>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
@@ -4151,12 +4209,12 @@
       </c>
       <c r="E48" s="8" t="inlineStr">
         <is>
-          <t>+$7.03K</t>
+          <t>+$59.72K</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>+$112.41K</t>
+          <t>+$144.03K</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
@@ -4169,40 +4227,36 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>4128.38</v>
+        <v>29522.6</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>83</v>
+        <v>29350</v>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>NDX</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t>+$33.55K</t>
+          <t>+$80.79K</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>+$110.46K</t>
+          <t>+$137.00K</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H49" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
@@ -4211,24 +4265,24 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>29272.6</v>
+        <v>29442.6</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>29100</v>
+        <v>29270</v>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E50" s="4" t="inlineStr">
-        <is>
-          <t>-$14.64K</t>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>+$7.03K</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>+$108.31K</t>
+          <t>+$112.41K</t>
         </is>
       </c>
       <c r="G50" s="3" t="inlineStr">
@@ -4241,43 +4295,115 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="n">
+        <v>4128.38</v>
+      </c>
+      <c r="C51" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>+$33.55K</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>+$110.46K</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B51" s="2" t="n">
+      <c r="B52" s="2" t="n">
+        <v>29272.6</v>
+      </c>
+      <c r="C52" s="2" t="n">
+        <v>29100</v>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>-$14.64K</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>+$108.31K</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="n">
         <v>29432.6</v>
       </c>
-      <c r="C51" s="2" t="n">
+      <c r="C53" s="2" t="n">
         <v>29260</v>
       </c>
-      <c r="D51" s="3" t="inlineStr">
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E51" s="4" t="inlineStr">
+      <c r="E53" s="4" t="inlineStr">
         <is>
           <t>-$80.79K</t>
         </is>
       </c>
-      <c r="F51" s="3" t="inlineStr">
+      <c r="F53" s="3" t="inlineStr">
         <is>
           <t>+$87.82K</t>
         </is>
       </c>
-      <c r="G51" s="3" t="inlineStr">
+      <c r="G53" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H51" s="3" t="inlineStr">
+      <c r="H53" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H51"/>
+  <autoFilter ref="A1:H53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>